<commit_message>
fix error, implement staff loan
</commit_message>
<xml_diff>
--- a/Sample Staff.xlsx
+++ b/Sample Staff.xlsx
@@ -5,22 +5,35 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myrp-my.sharepoint.com/personal/24042288_myrp_edu_sg/Documents/Backup/Year 3 Sem 1/FYP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\24042288\OneDrive - Republic Polytechnic\Backup\Year 3 Sem 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="186" documentId="8_{4D4153F6-E03A-4FD6-8B60-9B4A254272F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0B7678B-8916-4DBE-81BA-45DE023C0D43}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA88DC2-DCC2-4C53-8554-E55F29FC4856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{74950F5E-E29F-438F-837B-76CF067D30B2}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{74950F5E-E29F-438F-837B-76CF067D30B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Staff" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="60">
   <si>
     <t>email</t>
   </si>
@@ -112,9 +125,6 @@
     <t>Sarah Lim</t>
   </si>
   <si>
-    <t>Ahamd Razif</t>
-  </si>
-  <si>
     <t>Michelle Ong</t>
   </si>
   <si>
@@ -139,13 +149,70 @@
     <t>MichelleOng992@paynivo.com</t>
   </si>
   <si>
-    <t>Ahamd_Razi90f@paynivo.com</t>
-  </si>
-  <si>
     <t>Sarah2Lim@paynivo.com</t>
   </si>
   <si>
     <t>Jason.T@paynivo.com</t>
+  </si>
+  <si>
+    <t>race</t>
+  </si>
+  <si>
+    <t>religion</t>
+  </si>
+  <si>
+    <t>bank</t>
+  </si>
+  <si>
+    <t>account_no</t>
+  </si>
+  <si>
+    <t>Ahmad Razif</t>
+  </si>
+  <si>
+    <t>Ahmad_Razi90f@paynivo.com</t>
+  </si>
+  <si>
+    <t>Malay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chinese </t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>Islam</t>
+  </si>
+  <si>
+    <t>Indian</t>
+  </si>
+  <si>
+    <t>Hindu</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Christianity</t>
+  </si>
+  <si>
+    <t>Buddhism</t>
+  </si>
+  <si>
+    <t>POSB</t>
+  </si>
+  <si>
+    <t>Maybank</t>
+  </si>
+  <si>
+    <t>OCBC</t>
+  </si>
+  <si>
+    <t>DBS</t>
+  </si>
+  <si>
+    <t>UOB</t>
   </si>
 </sst>
 </file>
@@ -696,10 +763,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1019,10 +1082,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51825EF5-8265-44FA-B4D2-D3006E38C382}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="12.26953125" customWidth="1"/>
     <col min="2" max="2" width="22.6328125" customWidth="1"/>
     <col min="3" max="3" width="28.81640625" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
@@ -1032,11 +1095,12 @@
     <col min="9" max="9" width="14.54296875" customWidth="1"/>
     <col min="10" max="10" width="13.36328125" style="2" customWidth="1"/>
     <col min="11" max="11" width="12.54296875" customWidth="1"/>
+    <col min="15" max="15" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -1054,7 +1118,7 @@
         <v>12</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H1" t="s">
         <v>13</v>
@@ -1068,8 +1132,20 @@
       <c r="K1" t="s">
         <v>16</v>
       </c>
+      <c r="L1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N1" t="s">
+        <v>42</v>
+      </c>
+      <c r="O1" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1100,8 +1176,21 @@
       <c r="J2" s="2">
         <v>2</v>
       </c>
+      <c r="L2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" t="str">
+        <f ca="1">TEXT(RANDBETWEEN(100,999),"000")&amp;"-"&amp;TEXT(RANDBETWEEN(1000000,9999999),"0000000")&amp;"-"&amp;TEXT(RANDBETWEEN(0,9),"0")</f>
+        <v>222-6663034-3</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1132,13 +1221,26 @@
       <c r="J3" s="2">
         <v>2</v>
       </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" t="s">
+        <v>56</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O11" ca="1" si="0">TEXT(RANDBETWEEN(100,999),"000")&amp;"-"&amp;TEXT(RANDBETWEEN(1000000,9999999),"0000000")&amp;"-"&amp;TEXT(RANDBETWEEN(0,9),"0")</f>
+        <v>671-5148302-3</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -1164,8 +1266,21 @@
       <c r="J4" s="2">
         <v>2</v>
       </c>
+      <c r="L4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" t="s">
+        <v>57</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>150-6660936-1</v>
+      </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1175,7 +1290,7 @@
       <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
         <v>91234567</v>
       </c>
       <c r="E5" s="1">
@@ -1196,18 +1311,31 @@
       <c r="J5" s="2">
         <v>3</v>
       </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
+        <v>49</v>
+      </c>
+      <c r="N5" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>160-6441459-3</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6">
         <v>91234568</v>
       </c>
       <c r="E6" s="1">
@@ -1228,18 +1356,31 @@
       <c r="J6" s="2">
         <v>3</v>
       </c>
+      <c r="L6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M6" t="s">
+        <v>54</v>
+      </c>
+      <c r="N6" t="s">
+        <v>58</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>232-8505791-8</v>
+      </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="3">
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7">
         <v>91234569</v>
       </c>
       <c r="E7" s="1">
@@ -1260,18 +1401,31 @@
       <c r="J7" s="2">
         <v>4</v>
       </c>
+      <c r="L7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N7" t="s">
+        <v>57</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>956-7157488-0</v>
+      </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="3">
+        <v>45</v>
+      </c>
+      <c r="D8">
         <v>91234570</v>
       </c>
       <c r="E8" s="1">
@@ -1292,18 +1446,31 @@
       <c r="J8" s="2">
         <v>4</v>
       </c>
+      <c r="L8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N8" t="s">
+        <v>56</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>301-1282764-9</v>
+      </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="3">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9">
         <v>91234571</v>
       </c>
       <c r="E9" s="1">
@@ -1324,18 +1491,31 @@
       <c r="J9" s="2">
         <v>5</v>
       </c>
+      <c r="L9" t="s">
+        <v>47</v>
+      </c>
+      <c r="M9" t="s">
+        <v>52</v>
+      </c>
+      <c r="N9" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>127-1053892-2</v>
+      </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="3">
+        <v>35</v>
+      </c>
+      <c r="D10">
         <v>91234572</v>
       </c>
       <c r="E10" s="1">
@@ -1356,16 +1536,29 @@
       <c r="J10" s="2">
         <v>5</v>
       </c>
+      <c r="L10" t="s">
+        <v>47</v>
+      </c>
+      <c r="M10" t="s">
+        <v>53</v>
+      </c>
+      <c r="N10" t="s">
+        <v>59</v>
+      </c>
+      <c r="O10" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>859-3834759-8</v>
+      </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>26</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>37</v>
+      <c r="C11" t="s">
+        <v>36</v>
       </c>
       <c r="D11">
         <v>82364857</v>
@@ -1387,6 +1580,19 @@
       </c>
       <c r="J11" s="2">
         <v>6</v>
+      </c>
+      <c r="L11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N11" t="s">
+        <v>59</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>915-9675246-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>